<commit_message>
docs: refresh Fund Mapping Document after generator wording update
Regenerate only fund_structure.xlsx with the current rules mapdoc writer.
The Fund workbook arrived through #1003 with older Company wording before
#1009 generalized descriptions to each kind and refreshed the other workbooks.
Only Matching rules F2/F3 change; all other cells and Notes are preserved.

The existing catalog equality test reproduced the CI failure before this
regeneration. All 24 affected testmon tests pass after it. No rule, runtime
or test implementation changes. Track live PR verification in the ticket.
</commit_message>
<xml_diff>
--- a/rules/merge/kinds/fund_structure.xlsx
+++ b/rules/merge/kinds/fund_structure.xlsx
@@ -774,7 +774,7 @@
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>The record's SEC_SERIES_ID is the one a Company holds; and Exactly one Company holds that SEC_SERIES_ID, or none</t>
+          <t>The record's SEC_SERIES_ID is the one a Fund structure holds; and Exactly one Fund structure holds that SEC_SERIES_ID, or none</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -812,7 +812,7 @@
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>The record's LEI is the one a Company holds; and Exactly one Company holds that LEI, or none</t>
+          <t>The record's LEI is the one a Fund structure holds; and Exactly one Fund structure holds that LEI, or none</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -884,7 +884,7 @@
           <t>rules file comment</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -902,7 +902,7 @@
           <t>rules file comment</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -920,7 +920,7 @@
           <t>rules file comment</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -938,7 +938,7 @@
           <t>rules file comment</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr"/>
+      <c r="D5" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>